<commit_message>
added max token output to tesT.py, fixed bug in reading *adj.txt files
</commit_message>
<xml_diff>
--- a/Results Dataset 01 non-reasoning.xlsx
+++ b/Results Dataset 01 non-reasoning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valer\Documents\Master\Thesis\Scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AEE85E9-E7EB-44C5-BF74-3BE51C560765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F374F5-B0D5-4DDB-B629-09C5C0D4A15F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="6852" windowHeight="12336" xr2:uid="{A3AD4B4E-2473-4ED7-9538-EB5746896E87}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A3AD4B4E-2473-4ED7-9538-EB5746896E87}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
   <si>
     <t>2x2</t>
   </si>
@@ -126,6 +126,12 @@
   </si>
   <si>
     <t>tokenized occ</t>
+  </si>
+  <si>
+    <t>Complexity</t>
+  </si>
+  <si>
+    <t>beweegt voorbij doel</t>
   </si>
 </sst>
 </file>
@@ -155,7 +161,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -163,17 +169,205 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="13">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -184,6 +378,28 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{29DDA767-C800-4A8F-801C-D1CACC918AE9}" name="Table1" displayName="Table1" ref="A1:M4" totalsRowShown="0">
+  <autoFilter ref="A1:M4" xr:uid="{29DDA767-C800-4A8F-801C-D1CACC918AE9}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{4753E92D-E361-4C45-8B41-73AD6DE357ED}" name="Complexity" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{21B76EB6-F5AD-43B2-AD5D-FE513E5C6121}" name="JPG line" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{746D8278-0696-4561-B2E2-4BAB9BA9FA9D}" name="JSON line" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{FC1D4B5D-3FAB-4E35-AFFD-9F75B962EB1E}" name="adj JSON line" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{E17927AB-8C8C-4D89-8485-B843626F78AC}" name="adj txt line" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{BE4779C9-0B3F-47E0-852B-81F28F89FF72}" name="ASCII line" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{D4F54486-A17A-46DB-AA9B-DD949761775A}" name="tokenized line" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{FD450B04-53EF-4F99-9D16-483370ACB92B}" name="JPG occ" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{189C8E9B-5676-471B-9CE9-36E8D2E87B0C}" name="JSON occ" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{54155464-AD9C-46E7-B197-C9B8D6821A0A}" name="adj JSON occ" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{56D992AB-820A-4CB3-9F6E-2D1C64671203}" name="adj txt occ" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{57FB2F84-E603-44D6-86D5-A271FC3920E1}" name="ASCII occ" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{332C7BDD-7869-44B6-9D16-5EE6EDCCFACD}" name="tokenized occ" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -503,139 +719,426 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D99500E-C4D7-42C6-8284-189232F315D7}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" customWidth="1"/>
+    <col min="2" max="5" width="16.5546875" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" customWidth="1"/>
+    <col min="7" max="8" width="16.5546875" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" customWidth="1"/>
+    <col min="10" max="12" width="16.5546875" customWidth="1"/>
+    <col min="13" max="13" width="18.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B1" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="4" t="s">
         <v>21</v>
       </c>
       <c r="F1" t="s">
         <v>22</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4">
+        <v>0</v>
+      </c>
+      <c r="C2" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4">
+        <v>1</v>
+      </c>
+      <c r="K2" s="4">
+        <v>0</v>
+      </c>
+      <c r="L2" s="4">
+        <v>1</v>
+      </c>
+      <c r="M2" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="B4" s="4">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4">
+        <v>0</v>
+      </c>
+      <c r="M4" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+    </row>
+    <row r="7" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="10">
+        <v>0</v>
+      </c>
+      <c r="C7" s="10">
+        <v>1</v>
+      </c>
+      <c r="D7" s="10">
+        <v>0</v>
+      </c>
+      <c r="E7" s="10">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="10">
+        <v>0</v>
+      </c>
+      <c r="H7" s="10">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7" s="10">
+        <v>1</v>
+      </c>
+      <c r="K7" s="10">
+        <v>0</v>
+      </c>
+      <c r="L7" s="10">
+        <v>1</v>
+      </c>
+      <c r="M7" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+    </row>
+    <row r="8" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="8">
+        <v>0.33329999999999999</v>
+      </c>
+      <c r="C8" s="8">
+        <v>0.16669999999999999</v>
+      </c>
+      <c r="D8" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="F8" s="10">
+        <v>0</v>
+      </c>
+      <c r="G8" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="H8" s="8">
+        <v>0.16669999999999999</v>
+      </c>
+      <c r="I8" s="10">
+        <v>0</v>
+      </c>
+      <c r="J8" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="K8" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="L8" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="M8" s="11">
+        <v>0.33329999999999999</v>
+      </c>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="9">
+        <v>0.125</v>
+      </c>
+      <c r="C9" s="9">
+        <v>0.125</v>
+      </c>
+      <c r="D9" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="F9" s="9">
+        <v>0.125</v>
+      </c>
+      <c r="G9" s="9">
+        <v>0.125</v>
+      </c>
+      <c r="H9" s="9">
+        <v>0.125</v>
+      </c>
+      <c r="I9" s="7">
+        <v>0</v>
+      </c>
+      <c r="J9" s="9">
+        <v>0.125</v>
+      </c>
+      <c r="K9" s="9">
+        <v>0.1875</v>
+      </c>
+      <c r="L9" s="7">
+        <v>0</v>
+      </c>
+      <c r="M9" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>